<commit_message>
Registra precios finales de venta (para llevar / instalado)
El dueño definió los precios reales de venta, con dos tarifas por
repuesto instalable (para llevar vs instalado + mano de obra), en vez
del cálculo automático costo+19%+40%. Se documentan en 05-compras.md,
se agregan como columnas de referencia en el Excel del primer pedido, y
se deja la regla de dos tarifas como política de precio en
02-estrategia-comercial-marketing.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JaL6YE53y3yVJQXcbgPuCU
</commit_message>
<xml_diff>
--- a/empresa/compras/2026-09-12-primer-pedido.xlsx
+++ b/empresa/compras/2026-09-12-primer-pedido.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,6 +73,12 @@
       <name val="Arial"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001B5E20"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -118,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -150,6 +156,9 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -515,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -530,6 +539,8 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -607,6 +618,16 @@
           <t>Nota</t>
         </is>
       </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Precio final para llevar</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Precio final instalado</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -655,6 +676,14 @@
         <v>1</v>
       </c>
       <c r="L5" s="7" t="inlineStr"/>
+      <c r="M5" s="21" t="n">
+        <v>4500</v>
+      </c>
+      <c r="N5" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -703,6 +732,12 @@
         <v>3</v>
       </c>
       <c r="L6" s="7" t="inlineStr"/>
+      <c r="M6" s="21" t="n">
+        <v>18000</v>
+      </c>
+      <c r="N6" s="21" t="n">
+        <v>20000</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -751,6 +786,12 @@
         <v>3</v>
       </c>
       <c r="L7" s="7" t="inlineStr"/>
+      <c r="M7" s="21" t="n">
+        <v>18000</v>
+      </c>
+      <c r="N7" s="21" t="n">
+        <v>20000</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -799,6 +840,12 @@
         <v>1</v>
       </c>
       <c r="L8" s="7" t="inlineStr"/>
+      <c r="M8" s="21" t="n">
+        <v>18000</v>
+      </c>
+      <c r="N8" s="21" t="n">
+        <v>20000</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -847,6 +894,12 @@
         <v>3</v>
       </c>
       <c r="L9" s="7" t="inlineStr"/>
+      <c r="M9" s="21" t="n">
+        <v>18000</v>
+      </c>
+      <c r="N9" s="21" t="n">
+        <v>20000</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -895,6 +948,12 @@
         <v>3</v>
       </c>
       <c r="L10" s="7" t="inlineStr"/>
+      <c r="M10" s="21" t="n">
+        <v>70000</v>
+      </c>
+      <c r="N10" s="21" t="n">
+        <v>78000</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -943,6 +1002,12 @@
         <v>3</v>
       </c>
       <c r="L11" s="7" t="inlineStr"/>
+      <c r="M11" s="21" t="n">
+        <v>70000</v>
+      </c>
+      <c r="N11" s="21" t="n">
+        <v>78000</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -991,6 +1056,12 @@
         <v>1</v>
       </c>
       <c r="L12" s="7" t="inlineStr"/>
+      <c r="M12" s="21" t="n">
+        <v>70000</v>
+      </c>
+      <c r="N12" s="21" t="n">
+        <v>78000</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1039,6 +1110,12 @@
         <v>3</v>
       </c>
       <c r="L13" s="7" t="inlineStr"/>
+      <c r="M13" s="21" t="n">
+        <v>70000</v>
+      </c>
+      <c r="N13" s="21" t="n">
+        <v>78000</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -1091,6 +1168,12 @@
           <t>Codigo original del proveedor (KIT-AKT0) duplicado con el de la fila 7 - se le asigno un codigo distinto</t>
         </is>
       </c>
+      <c r="M14" s="21" t="n">
+        <v>70000</v>
+      </c>
+      <c r="N14" s="21" t="n">
+        <v>78000</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1139,6 +1222,12 @@
         <v>1</v>
       </c>
       <c r="L15" s="7" t="inlineStr"/>
+      <c r="M15" s="21" t="n">
+        <v>70000</v>
+      </c>
+      <c r="N15" s="21" t="n">
+        <v>78000</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1187,6 +1276,12 @@
         <v>3</v>
       </c>
       <c r="L16" s="7" t="inlineStr"/>
+      <c r="M16" s="21" t="n">
+        <v>20000</v>
+      </c>
+      <c r="N16" s="21" t="n">
+        <v>24900</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1235,6 +1330,14 @@
         <v>3</v>
       </c>
       <c r="L17" s="7" t="inlineStr"/>
+      <c r="M17" s="21" t="n">
+        <v>8500</v>
+      </c>
+      <c r="N17" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1283,6 +1386,14 @@
         <v>3</v>
       </c>
       <c r="L18" s="7" t="inlineStr"/>
+      <c r="M18" s="21" t="n">
+        <v>8500</v>
+      </c>
+      <c r="N18" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1331,6 +1442,14 @@
         <v>3</v>
       </c>
       <c r="L19" s="7" t="inlineStr"/>
+      <c r="M19" s="21" t="n">
+        <v>18000</v>
+      </c>
+      <c r="N19" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1379,6 +1498,14 @@
         <v>3</v>
       </c>
       <c r="L20" s="7" t="inlineStr"/>
+      <c r="M20" s="21" t="n">
+        <v>18000</v>
+      </c>
+      <c r="N20" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1427,6 +1554,14 @@
         <v>3</v>
       </c>
       <c r="L21" s="7" t="inlineStr"/>
+      <c r="M21" s="21" t="n">
+        <v>18000</v>
+      </c>
+      <c r="N21" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1475,6 +1610,12 @@
         <v>3</v>
       </c>
       <c r="L22" s="7" t="inlineStr"/>
+      <c r="M22" s="21" t="n">
+        <v>20000</v>
+      </c>
+      <c r="N22" s="21" t="n">
+        <v>24000</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
@@ -1525,6 +1666,14 @@
       <c r="L23" s="11" t="inlineStr">
         <is>
           <t>Cantidad y precio escritos a mano y dificiles de leer - CONFIRMAR con el proveedor antes de dar por buena esta fila</t>
+        </is>
+      </c>
+      <c r="M23" s="21" t="n">
+        <v>8500</v>
+      </c>
+      <c r="N23" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -1555,8 +1704,54 @@
       <c r="K24" s="12" t="n"/>
       <c r="L24" s="12" t="n"/>
     </row>
+    <row r="25">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>TRO-RESORTE</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>Resorte de trompo stop (suelto, repuesto aparte)</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="inlineStr">
+        <is>
+          <t>Varios</t>
+        </is>
+      </c>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
+          <t>Premium Racing</t>
+        </is>
+      </c>
+      <c r="E25" s="22" t="n"/>
+      <c r="F25" s="22" t="n"/>
+      <c r="G25" s="22" t="n"/>
+      <c r="H25" s="22" t="n"/>
+      <c r="I25" s="22" t="n"/>
+      <c r="J25" s="22" t="n"/>
+      <c r="K25" s="22" t="n"/>
+      <c r="L25" s="22" t="inlineStr">
+        <is>
+          <t>Sale de las mismas unidades de TRO-PAQU; no es un producto comprado aparte, es el mismo resorte vendido suelto.</t>
+        </is>
+      </c>
+      <c r="M25" s="23" t="n">
+        <v>1500</v>
+      </c>
+      <c r="N25" s="22" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Precios finales (M, N) definidos por el dueño el 17/09/2026 - reemplazan el calculo automatico de la columna H para decisiones de venta reales.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A27:N27"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A1:L1"/>
   </mergeCells>

</xml_diff>